<commit_message>
Fix Excel reading and plotting workflow
</commit_message>
<xml_diff>
--- a/Results/EmissionsByProd.xlsx
+++ b/Results/EmissionsByProd.xlsx
@@ -938,10 +938,10 @@
         <v>182</v>
       </c>
       <c r="D16" t="n">
-        <v>9.62268519939735</v>
+        <v>9.610226459166865</v>
       </c>
       <c r="E16" t="n">
-        <v>1.2874693461898898</v>
+        <v>1.2823973599864067</v>
       </c>
       <c r="F16" t="s">
         <v>186</v>
@@ -958,10 +958,10 @@
         <v>182</v>
       </c>
       <c r="D17" t="n">
-        <v>9.642061335952905</v>
+        <v>9.628180796923965</v>
       </c>
       <c r="E17" t="n">
-        <v>1.2880860538347816</v>
+        <v>1.285859753233072</v>
       </c>
       <c r="F17" t="s">
         <v>186</v>
@@ -978,10 +978,10 @@
         <v>182</v>
       </c>
       <c r="D18" t="n">
-        <v>9.611560041565784</v>
+        <v>9.61957495015523</v>
       </c>
       <c r="E18" t="n">
-        <v>1.2873698291281992</v>
+        <v>1.3031675810944305</v>
       </c>
       <c r="F18" t="s">
         <v>186</v>
@@ -998,10 +998,10 @@
         <v>182</v>
       </c>
       <c r="D19" t="n">
-        <v>9.43360198202779</v>
+        <v>9.42731534849362</v>
       </c>
       <c r="E19" t="n">
-        <v>1.2691608505691527</v>
+        <v>1.2870033353327612</v>
       </c>
       <c r="F19" t="s">
         <v>186</v>
@@ -1018,10 +1018,10 @@
         <v>182</v>
       </c>
       <c r="D20" t="n">
-        <v>11.222010784020974</v>
+        <v>11.222017447138299</v>
       </c>
       <c r="E20" t="n">
-        <v>1.4975077541036979</v>
+        <v>1.4939627362728836</v>
       </c>
       <c r="F20" t="s">
         <v>186</v>
@@ -1038,10 +1038,10 @@
         <v>182</v>
       </c>
       <c r="D21" t="n">
-        <v>11.448354502316135</v>
+        <v>11.444080430116703</v>
       </c>
       <c r="E21" t="n">
-        <v>1.5127566402261983</v>
+        <v>1.515832450080378</v>
       </c>
       <c r="F21" t="s">
         <v>186</v>
@@ -1058,10 +1058,10 @@
         <v>182</v>
       </c>
       <c r="D22" t="n">
-        <v>11.243023910581076</v>
+        <v>11.247602650474247</v>
       </c>
       <c r="E22" t="n">
-        <v>1.4884317779263627</v>
+        <v>1.4986110995782662</v>
       </c>
       <c r="F22" t="s">
         <v>186</v>
@@ -1078,10 +1078,10 @@
         <v>183</v>
       </c>
       <c r="D23" t="n">
-        <v>25.92660400518055</v>
+        <v>25.876864680978386</v>
       </c>
       <c r="E23" t="n">
-        <v>5.61450736937615</v>
+        <v>5.61425739287497</v>
       </c>
       <c r="F23" t="s">
         <v>186</v>
@@ -1098,10 +1098,10 @@
         <v>183</v>
       </c>
       <c r="D24" t="n">
-        <v>25.836937324429673</v>
+        <v>25.905769234664533</v>
       </c>
       <c r="E24" t="n">
-        <v>5.615399846870188</v>
+        <v>5.575980477865198</v>
       </c>
       <c r="F24" t="s">
         <v>186</v>
@@ -1118,10 +1118,10 @@
         <v>183</v>
       </c>
       <c r="D25" t="n">
-        <v>25.788771055372745</v>
+        <v>25.837483806484407</v>
       </c>
       <c r="E25" t="n">
-        <v>5.5842940848299945</v>
+        <v>5.563900233608715</v>
       </c>
       <c r="F25" t="s">
         <v>186</v>
@@ -1138,10 +1138,10 @@
         <v>183</v>
       </c>
       <c r="D26" t="n">
-        <v>25.9479453480757</v>
+        <v>25.846114374221436</v>
       </c>
       <c r="E26" t="n">
-        <v>5.57724449169959</v>
+        <v>5.584470896888371</v>
       </c>
       <c r="F26" t="s">
         <v>186</v>
@@ -1158,10 +1158,10 @@
         <v>183</v>
       </c>
       <c r="D27" t="n">
-        <v>31.870634160649594</v>
+        <v>31.81397705343757</v>
       </c>
       <c r="E27" t="n">
-        <v>6.5961389773129655</v>
+        <v>6.47531637549404</v>
       </c>
       <c r="F27" t="s">
         <v>186</v>
@@ -1178,10 +1178,10 @@
         <v>183</v>
       </c>
       <c r="D28" t="n">
-        <v>31.735439353284814</v>
+        <v>31.818570405098384</v>
       </c>
       <c r="E28" t="n">
-        <v>6.56326981531616</v>
+        <v>6.481632613450441</v>
       </c>
       <c r="F28" t="s">
         <v>186</v>
@@ -1198,10 +1198,10 @@
         <v>183</v>
       </c>
       <c r="D29" t="n">
-        <v>31.71172462337099</v>
+        <v>31.752961492582838</v>
       </c>
       <c r="E29" t="n">
-        <v>6.424015695770721</v>
+        <v>6.587545891143051</v>
       </c>
       <c r="F29" t="s">
         <v>186</v>
@@ -1218,10 +1218,10 @@
         <v>184</v>
       </c>
       <c r="D30" t="n">
-        <v>71.37985401891225</v>
+        <v>71.5801448109893</v>
       </c>
       <c r="E30" t="n">
-        <v>14.693824220391923</v>
+        <v>14.516226924716488</v>
       </c>
       <c r="F30" t="s">
         <v>186</v>
@@ -1238,10 +1238,10 @@
         <v>184</v>
       </c>
       <c r="D31" t="n">
-        <v>71.15976577945158</v>
+        <v>71.3678454094877</v>
       </c>
       <c r="E31" t="n">
-        <v>14.536856584124093</v>
+        <v>14.552223865419139</v>
       </c>
       <c r="F31" t="s">
         <v>186</v>
@@ -1258,10 +1258,10 @@
         <v>184</v>
       </c>
       <c r="D32" t="n">
-        <v>71.41865046868404</v>
+        <v>71.16590622061615</v>
       </c>
       <c r="E32" t="n">
-        <v>14.4703433189328</v>
+        <v>14.49389676910977</v>
       </c>
       <c r="F32" t="s">
         <v>186</v>
@@ -1278,10 +1278,10 @@
         <v>184</v>
       </c>
       <c r="D33" t="n">
-        <v>89.44736176694066</v>
+        <v>89.1993485504792</v>
       </c>
       <c r="E33" t="n">
-        <v>18.30549797131276</v>
+        <v>18.172675709518227</v>
       </c>
       <c r="F33" t="s">
         <v>186</v>
@@ -1298,10 +1298,10 @@
         <v>184</v>
       </c>
       <c r="D34" t="n">
-        <v>103.8195198643172</v>
+        <v>103.72713418822242</v>
       </c>
       <c r="E34" t="n">
-        <v>21.069642264478627</v>
+        <v>20.913034590399782</v>
       </c>
       <c r="F34" t="s">
         <v>186</v>
@@ -1318,10 +1318,10 @@
         <v>184</v>
       </c>
       <c r="D35" t="n">
-        <v>103.86056140654794</v>
+        <v>104.06321236827657</v>
       </c>
       <c r="E35" t="n">
-        <v>21.077689538671713</v>
+        <v>21.00403156638593</v>
       </c>
       <c r="F35" t="s">
         <v>186</v>
@@ -1338,10 +1338,10 @@
         <v>184</v>
       </c>
       <c r="D36" t="n">
-        <v>103.7164597672051</v>
+        <v>103.89239042902058</v>
       </c>
       <c r="E36" t="n">
-        <v>20.89038531900938</v>
+        <v>20.773606913800517</v>
       </c>
       <c r="F36" t="s">
         <v>186</v>
@@ -1358,10 +1358,10 @@
         <v>185</v>
       </c>
       <c r="D37" t="n">
-        <v>214.23777773627145</v>
+        <v>213.26802273131636</v>
       </c>
       <c r="E37" t="n">
-        <v>39.51104022563772</v>
+        <v>39.00773078574014</v>
       </c>
       <c r="F37" t="s">
         <v>186</v>
@@ -1378,10 +1378,10 @@
         <v>185</v>
       </c>
       <c r="D38" t="n">
-        <v>214.30565365288095</v>
+        <v>214.60642870760844</v>
       </c>
       <c r="E38" t="n">
-        <v>39.40664799943641</v>
+        <v>39.239340574570434</v>
       </c>
       <c r="F38" t="s">
         <v>186</v>
@@ -1398,10 +1398,10 @@
         <v>185</v>
       </c>
       <c r="D39" t="n">
-        <v>213.95043526567096</v>
+        <v>214.0550446806084</v>
       </c>
       <c r="E39" t="n">
-        <v>38.98082454647248</v>
+        <v>39.436228652126104</v>
       </c>
       <c r="F39" t="s">
         <v>186</v>
@@ -1418,10 +1418,10 @@
         <v>185</v>
       </c>
       <c r="D40" t="n">
-        <v>178.35239385323192</v>
+        <v>177.99897888810727</v>
       </c>
       <c r="E40" t="n">
-        <v>34.750427357282184</v>
+        <v>34.679208437879716</v>
       </c>
       <c r="F40" t="s">
         <v>186</v>
@@ -1438,10 +1438,10 @@
         <v>185</v>
       </c>
       <c r="D41" t="n">
-        <v>207.696739802068</v>
+        <v>208.14634944882962</v>
       </c>
       <c r="E41" t="n">
-        <v>39.93733576027936</v>
+        <v>40.379344873541214</v>
       </c>
       <c r="F41" t="s">
         <v>186</v>
@@ -1458,10 +1458,10 @@
         <v>185</v>
       </c>
       <c r="D42" t="n">
-        <v>206.9060210293444</v>
+        <v>207.47869740409504</v>
       </c>
       <c r="E42" t="n">
-        <v>39.77283699379192</v>
+        <v>40.19588250922482</v>
       </c>
       <c r="F42" t="s">
         <v>186</v>
@@ -1478,10 +1478,10 @@
         <v>185</v>
       </c>
       <c r="D43" t="n">
-        <v>207.05533733632345</v>
+        <v>207.25803407064384</v>
       </c>
       <c r="E43" t="n">
-        <v>40.046769220218195</v>
+        <v>40.34888537912307</v>
       </c>
       <c r="F43" t="s">
         <v>186</v>
@@ -2058,10 +2058,10 @@
         <v>184</v>
       </c>
       <c r="D72" t="n">
-        <v>7.127142457488263</v>
+        <v>7.151723488811559</v>
       </c>
       <c r="E72" t="n">
-        <v>1.8298310128709077</v>
+        <v>1.8296503420066792</v>
       </c>
       <c r="F72" t="s">
         <v>187</v>
@@ -2078,10 +2078,10 @@
         <v>184</v>
       </c>
       <c r="D73" t="n">
-        <v>7.126033802215482</v>
+        <v>7.1259291789966515</v>
       </c>
       <c r="E73" t="n">
-        <v>1.855564348615052</v>
+        <v>1.8245798460509424</v>
       </c>
       <c r="F73" t="s">
         <v>187</v>
@@ -2098,10 +2098,10 @@
         <v>184</v>
       </c>
       <c r="D74" t="n">
-        <v>7.113272265182493</v>
+        <v>7.1327051713116</v>
       </c>
       <c r="E74" t="n">
-        <v>1.8349981981018006</v>
+        <v>1.8255944723134339</v>
       </c>
       <c r="F74" t="s">
         <v>187</v>
@@ -2118,10 +2118,10 @@
         <v>184</v>
       </c>
       <c r="D75" t="n">
-        <v>17.807274936635274</v>
+        <v>17.79873877062355</v>
       </c>
       <c r="E75" t="n">
-        <v>4.535894658265783</v>
+        <v>4.5666640053812735</v>
       </c>
       <c r="F75" t="s">
         <v>187</v>
@@ -2138,10 +2138,10 @@
         <v>184</v>
       </c>
       <c r="D76" t="n">
-        <v>20.77916816592116</v>
+        <v>20.719354688942783</v>
       </c>
       <c r="E76" t="n">
-        <v>5.288020960074454</v>
+        <v>5.244261729762454</v>
       </c>
       <c r="F76" t="s">
         <v>187</v>
@@ -2158,10 +2158,10 @@
         <v>184</v>
       </c>
       <c r="D77" t="n">
-        <v>10.353090270698964</v>
+        <v>10.41346931040527</v>
       </c>
       <c r="E77" t="n">
-        <v>2.6454794309003025</v>
+        <v>2.6618036852685503</v>
       </c>
       <c r="F77" t="s">
         <v>187</v>
@@ -2178,10 +2178,10 @@
         <v>184</v>
       </c>
       <c r="D78" t="n">
-        <v>20.785672544026482</v>
+        <v>20.657268228760355</v>
       </c>
       <c r="E78" t="n">
-        <v>5.261518190404501</v>
+        <v>5.219398627437371</v>
       </c>
       <c r="F78" t="s">
         <v>187</v>
@@ -2198,10 +2198,10 @@
         <v>182</v>
       </c>
       <c r="D79" t="n">
-        <v>47.60055455166188</v>
+        <v>47.534558030230365</v>
       </c>
       <c r="E79" t="n">
-        <v>8.14187983172928</v>
+        <v>7.971085966055013</v>
       </c>
       <c r="F79" t="s">
         <v>187</v>
@@ -2218,10 +2218,10 @@
         <v>182</v>
       </c>
       <c r="D80" t="n">
-        <v>47.74118731959252</v>
+        <v>47.6779797634074</v>
       </c>
       <c r="E80" t="n">
-        <v>8.16464901834342</v>
+        <v>8.117196533635086</v>
       </c>
       <c r="F80" t="s">
         <v>187</v>
@@ -2238,10 +2238,10 @@
         <v>182</v>
       </c>
       <c r="D81" t="n">
-        <v>47.52746860158583</v>
+        <v>47.619801090564756</v>
       </c>
       <c r="E81" t="n">
-        <v>8.021019049796104</v>
+        <v>8.154260944352986</v>
       </c>
       <c r="F81" t="s">
         <v>187</v>
@@ -2258,10 +2258,10 @@
         <v>182</v>
       </c>
       <c r="D82" t="n">
-        <v>46.708920995705014</v>
+        <v>46.67095020386493</v>
       </c>
       <c r="E82" t="n">
-        <v>8.083217851708984</v>
+        <v>8.034600397205956</v>
       </c>
       <c r="F82" t="s">
         <v>187</v>
@@ -2278,10 +2278,10 @@
         <v>182</v>
       </c>
       <c r="D83" t="n">
-        <v>54.09787174422669</v>
+        <v>54.30908592534083</v>
       </c>
       <c r="E83" t="n">
-        <v>9.012360042820974</v>
+        <v>9.282631818605756</v>
       </c>
       <c r="F83" t="s">
         <v>187</v>
@@ -2298,10 +2298,10 @@
         <v>182</v>
       </c>
       <c r="D84" t="n">
-        <v>55.41775661329827</v>
+        <v>55.2622046998122</v>
       </c>
       <c r="E84" t="n">
-        <v>9.429003381178436</v>
+        <v>9.34245470860538</v>
       </c>
       <c r="F84" t="s">
         <v>187</v>
@@ -2318,10 +2318,10 @@
         <v>182</v>
       </c>
       <c r="D85" t="n">
-        <v>54.30999885175245</v>
+        <v>54.14824970967028</v>
       </c>
       <c r="E85" t="n">
-        <v>9.241628393186902</v>
+        <v>9.173039987963989</v>
       </c>
       <c r="F85" t="s">
         <v>187</v>
@@ -2478,10 +2478,10 @@
         <v>182</v>
       </c>
       <c r="D93" t="n">
-        <v>9.619798134106702</v>
+        <v>9.62085286320759</v>
       </c>
       <c r="E93" t="n">
-        <v>1.2871400493843372</v>
+        <v>1.2916427872513936</v>
       </c>
       <c r="F93" t="s">
         <v>188</v>
@@ -2498,10 +2498,10 @@
         <v>182</v>
       </c>
       <c r="D94" t="n">
-        <v>9.641436823174777</v>
+        <v>9.627162459856448</v>
       </c>
       <c r="E94" t="n">
-        <v>1.3025480718807674</v>
+        <v>1.2829732788923658</v>
       </c>
       <c r="F94" t="s">
         <v>188</v>
@@ -2518,10 +2518,10 @@
         <v>182</v>
       </c>
       <c r="D95" t="n">
-        <v>9.605301813220073</v>
+        <v>9.603117363500582</v>
       </c>
       <c r="E95" t="n">
-        <v>1.285377526880543</v>
+        <v>1.287573335107398</v>
       </c>
       <c r="F95" t="s">
         <v>188</v>
@@ -2538,10 +2538,10 @@
         <v>182</v>
       </c>
       <c r="D96" t="n">
-        <v>9.461408532926376</v>
+        <v>9.430300511924987</v>
       </c>
       <c r="E96" t="n">
-        <v>1.2878710371215516</v>
+        <v>1.2909342274742466</v>
       </c>
       <c r="F96" t="s">
         <v>188</v>
@@ -2558,10 +2558,10 @@
         <v>182</v>
       </c>
       <c r="D97" t="n">
-        <v>11.235657596563493</v>
+        <v>11.257479853231164</v>
       </c>
       <c r="E97" t="n">
-        <v>1.480927680972921</v>
+        <v>1.4835650961192342</v>
       </c>
       <c r="F97" t="s">
         <v>188</v>
@@ -2578,10 +2578,10 @@
         <v>182</v>
       </c>
       <c r="D98" t="n">
-        <v>11.455330552298383</v>
+        <v>11.43110260387498</v>
       </c>
       <c r="E98" t="n">
-        <v>1.4949234192865464</v>
+        <v>1.5084126239788722</v>
       </c>
       <c r="F98" t="s">
         <v>188</v>
@@ -2598,10 +2598,10 @@
         <v>182</v>
       </c>
       <c r="D99" t="n">
-        <v>11.23532469735653</v>
+        <v>11.237943077429847</v>
       </c>
       <c r="E99" t="n">
-        <v>1.487041582957306</v>
+        <v>1.4937808241992088</v>
       </c>
       <c r="F99" t="s">
         <v>188</v>
@@ -2618,10 +2618,10 @@
         <v>183</v>
       </c>
       <c r="D100" t="n">
-        <v>12.979995262656104</v>
+        <v>13.004944059743728</v>
       </c>
       <c r="E100" t="n">
-        <v>2.8273479971979025</v>
+        <v>2.8095973069772566</v>
       </c>
       <c r="F100" t="s">
         <v>188</v>
@@ -2638,10 +2638,10 @@
         <v>183</v>
       </c>
       <c r="D101" t="n">
-        <v>12.913107979107977</v>
+        <v>12.964415061897013</v>
       </c>
       <c r="E101" t="n">
-        <v>2.798799866133791</v>
+        <v>2.783964352316294</v>
       </c>
       <c r="F101" t="s">
         <v>188</v>
@@ -2658,10 +2658,10 @@
         <v>183</v>
       </c>
       <c r="D102" t="n">
-        <v>12.99988146185089</v>
+        <v>12.96608148331707</v>
       </c>
       <c r="E102" t="n">
-        <v>2.7716291952124226</v>
+        <v>2.8219897732899972</v>
       </c>
       <c r="F102" t="s">
         <v>188</v>
@@ -2678,10 +2678,10 @@
         <v>183</v>
       </c>
       <c r="D103" t="n">
-        <v>12.939388063736216</v>
+        <v>12.89210817335776</v>
       </c>
       <c r="E103" t="n">
-        <v>2.798377494251825</v>
+        <v>2.7867715587183666</v>
       </c>
       <c r="F103" t="s">
         <v>188</v>
@@ -2698,10 +2698,10 @@
         <v>183</v>
       </c>
       <c r="D104" t="n">
-        <v>15.867160895490555</v>
+        <v>15.961037562000506</v>
       </c>
       <c r="E104" t="n">
-        <v>3.226178067454427</v>
+        <v>3.2550353276261537</v>
       </c>
       <c r="F104" t="s">
         <v>188</v>
@@ -2718,10 +2718,10 @@
         <v>183</v>
       </c>
       <c r="D105" t="n">
-        <v>15.949403246811391</v>
+        <v>15.79139566346463</v>
       </c>
       <c r="E105" t="n">
-        <v>3.2522233060001917</v>
+        <v>3.2256130159577587</v>
       </c>
       <c r="F105" t="s">
         <v>188</v>
@@ -2738,10 +2738,10 @@
         <v>183</v>
       </c>
       <c r="D106" t="n">
-        <v>15.849773324759182</v>
+        <v>15.943190993010774</v>
       </c>
       <c r="E106" t="n">
-        <v>3.255580873321123</v>
+        <v>3.2974563682553506</v>
       </c>
       <c r="F106" t="s">
         <v>188</v>
@@ -2758,10 +2758,10 @@
         <v>185</v>
       </c>
       <c r="D107" t="n">
-        <v>214.55391326602887</v>
+        <v>213.42215442054206</v>
       </c>
       <c r="E107" t="n">
-        <v>39.75886178039442</v>
+        <v>39.413964030599494</v>
       </c>
       <c r="F107" t="s">
         <v>188</v>
@@ -2778,10 +2778,10 @@
         <v>185</v>
       </c>
       <c r="D108" t="n">
-        <v>213.9961174458567</v>
+        <v>214.6219724939549</v>
       </c>
       <c r="E108" t="n">
-        <v>39.34199205884485</v>
+        <v>39.691013021635776</v>
       </c>
       <c r="F108" t="s">
         <v>188</v>
@@ -2798,10 +2798,10 @@
         <v>185</v>
       </c>
       <c r="D109" t="n">
-        <v>213.89755828309862</v>
+        <v>214.28321752275517</v>
       </c>
       <c r="E109" t="n">
-        <v>39.12704235768513</v>
+        <v>39.30432307921011</v>
       </c>
       <c r="F109" t="s">
         <v>188</v>
@@ -2818,10 +2818,10 @@
         <v>185</v>
       </c>
       <c r="D110" t="n">
-        <v>178.76982256722408</v>
+        <v>178.22932313504035</v>
       </c>
       <c r="E110" t="n">
-        <v>34.7391121609539</v>
+        <v>34.484297252548465</v>
       </c>
       <c r="F110" t="s">
         <v>188</v>
@@ -2838,10 +2838,10 @@
         <v>185</v>
       </c>
       <c r="D111" t="n">
-        <v>208.0830488381537</v>
+        <v>208.20268127042718</v>
       </c>
       <c r="E111" t="n">
-        <v>39.55715808448442</v>
+        <v>40.335626024827825</v>
       </c>
       <c r="F111" t="s">
         <v>188</v>
@@ -2858,10 +2858,10 @@
         <v>185</v>
       </c>
       <c r="D112" t="n">
-        <v>207.446074305974</v>
+        <v>206.6353101654328</v>
       </c>
       <c r="E112" t="n">
-        <v>40.20821360454722</v>
+        <v>39.84823846623577</v>
       </c>
       <c r="F112" t="s">
         <v>188</v>
@@ -2878,10 +2878,10 @@
         <v>185</v>
       </c>
       <c r="D113" t="n">
-        <v>207.3639666495104</v>
+        <v>208.02930726539373</v>
       </c>
       <c r="E113" t="n">
-        <v>40.22251269670122</v>
+        <v>40.57162313013321</v>
       </c>
       <c r="F113" t="s">
         <v>188</v>
@@ -2898,10 +2898,10 @@
         <v>181</v>
       </c>
       <c r="D114" t="n">
-        <v>285.82398289530454</v>
+        <v>285.52181105827646</v>
       </c>
       <c r="E114" t="n">
-        <v>55.53222124879974</v>
+        <v>55.08094459978561</v>
       </c>
       <c r="F114" t="s">
         <v>188</v>
@@ -2918,10 +2918,10 @@
         <v>181</v>
       </c>
       <c r="D115" t="n">
-        <v>285.2239231148237</v>
+        <v>285.63166774763647</v>
       </c>
       <c r="E115" t="n">
-        <v>55.037178755952645</v>
+        <v>55.391593519607135</v>
       </c>
       <c r="F115" t="s">
         <v>188</v>
@@ -2938,10 +2938,10 @@
         <v>181</v>
       </c>
       <c r="D116" t="n">
-        <v>285.14290271893594</v>
+        <v>284.3234745803618</v>
       </c>
       <c r="E116" t="n">
-        <v>55.093857058764</v>
+        <v>55.25471710611768</v>
       </c>
       <c r="F116" t="s">
         <v>188</v>
@@ -2958,10 +2958,10 @@
         <v>181</v>
       </c>
       <c r="D117" t="n">
-        <v>238.70136124712386</v>
+        <v>237.35921436145026</v>
       </c>
       <c r="E117" t="n">
-        <v>48.76822923622589</v>
+        <v>48.54887041851056</v>
       </c>
       <c r="F117" t="s">
         <v>188</v>
@@ -2978,10 +2978,10 @@
         <v>181</v>
       </c>
       <c r="D118" t="n">
-        <v>275.7203017530348</v>
+        <v>276.6163989226981</v>
       </c>
       <c r="E118" t="n">
-        <v>54.98140207622486</v>
+        <v>55.19902960362711</v>
       </c>
       <c r="F118" t="s">
         <v>188</v>
@@ -2998,10 +2998,10 @@
         <v>181</v>
       </c>
       <c r="D119" t="n">
-        <v>276.56427445804457</v>
+        <v>276.2375115357231</v>
       </c>
       <c r="E119" t="n">
-        <v>55.75235230912927</v>
+        <v>55.98517041534139</v>
       </c>
       <c r="F119" t="s">
         <v>188</v>
@@ -3018,10 +3018,10 @@
         <v>181</v>
       </c>
       <c r="D120" t="n">
-        <v>276.9671606795994</v>
+        <v>276.1658394202678</v>
       </c>
       <c r="E120" t="n">
-        <v>56.26829737625429</v>
+        <v>56.21231330911427</v>
       </c>
       <c r="F120" t="s">
         <v>188</v>
@@ -3038,10 +3038,10 @@
         <v>180</v>
       </c>
       <c r="D121" t="n">
-        <v>335.93158516781415</v>
+        <v>334.56970781331705</v>
       </c>
       <c r="E121" t="n">
-        <v>146.13152910805377</v>
+        <v>145.16051789111907</v>
       </c>
       <c r="F121" t="s">
         <v>188</v>
@@ -3058,10 +3058,10 @@
         <v>180</v>
       </c>
       <c r="D122" t="n">
-        <v>330.95888352284044</v>
+        <v>332.24801684814395</v>
       </c>
       <c r="E122" t="n">
-        <v>144.91523863494936</v>
+        <v>146.17490878694028</v>
       </c>
       <c r="F122" t="s">
         <v>188</v>
@@ -3078,10 +3078,10 @@
         <v>180</v>
       </c>
       <c r="D123" t="n">
-        <v>333.37881291461247</v>
+        <v>332.4628640488131</v>
       </c>
       <c r="E123" t="n">
-        <v>145.60960067726657</v>
+        <v>144.57972170208797</v>
       </c>
       <c r="F123" t="s">
         <v>188</v>
@@ -3098,10 +3098,10 @@
         <v>180</v>
       </c>
       <c r="D124" t="n">
-        <v>416.7364864299192</v>
+        <v>414.5022489661659</v>
       </c>
       <c r="E124" t="n">
-        <v>180.4218221025394</v>
+        <v>180.4341720155783</v>
       </c>
       <c r="F124" t="s">
         <v>188</v>
@@ -3118,10 +3118,10 @@
         <v>180</v>
       </c>
       <c r="D125" t="n">
-        <v>487.3415140790231</v>
+        <v>486.9945114109325</v>
       </c>
       <c r="E125" t="n">
-        <v>210.73496709920605</v>
+        <v>207.98846168133082</v>
       </c>
       <c r="F125" t="s">
         <v>188</v>
@@ -3138,10 +3138,10 @@
         <v>180</v>
       </c>
       <c r="D126" t="n">
-        <v>482.93024978418714</v>
+        <v>486.37473290304666</v>
       </c>
       <c r="E126" t="n">
-        <v>210.93880314093906</v>
+        <v>207.96965475657404</v>
       </c>
       <c r="F126" t="s">
         <v>188</v>
@@ -3158,10 +3158,10 @@
         <v>180</v>
       </c>
       <c r="D127" t="n">
-        <v>486.05572076391985</v>
+        <v>485.54531020836293</v>
       </c>
       <c r="E127" t="n">
-        <v>210.05559479548822</v>
+        <v>213.06586161480183</v>
       </c>
       <c r="F127" t="s">
         <v>188</v>
@@ -3738,10 +3738,10 @@
         <v>184</v>
       </c>
       <c r="D156" t="n">
-        <v>7.135691212258179</v>
+        <v>7.16527220434356</v>
       </c>
       <c r="E156" t="n">
-        <v>1.8215694825405038</v>
+        <v>1.8487035269813357</v>
       </c>
       <c r="F156" t="s">
         <v>189</v>
@@ -3758,10 +3758,10 @@
         <v>184</v>
       </c>
       <c r="D157" t="n">
-        <v>7.0987956117636495</v>
+        <v>7.13434540933927</v>
       </c>
       <c r="E157" t="n">
-        <v>1.834188994374235</v>
+        <v>1.8533647965843991</v>
       </c>
       <c r="F157" t="s">
         <v>189</v>
@@ -3778,10 +3778,10 @@
         <v>184</v>
       </c>
       <c r="D158" t="n">
-        <v>7.114482765220117</v>
+        <v>7.121828345492598</v>
       </c>
       <c r="E158" t="n">
-        <v>1.8276966487062354</v>
+        <v>1.8336484217703342</v>
       </c>
       <c r="F158" t="s">
         <v>189</v>
@@ -3798,10 +3798,10 @@
         <v>184</v>
       </c>
       <c r="D159" t="n">
-        <v>17.85715250051784</v>
+        <v>17.81394932679788</v>
       </c>
       <c r="E159" t="n">
-        <v>4.5844317296332235</v>
+        <v>4.553009048993307</v>
       </c>
       <c r="F159" t="s">
         <v>189</v>
@@ -3818,10 +3818,10 @@
         <v>184</v>
       </c>
       <c r="D160" t="n">
-        <v>20.776616775832398</v>
+        <v>20.764405836094088</v>
       </c>
       <c r="E160" t="n">
-        <v>5.336510765683969</v>
+        <v>5.347387562041506</v>
       </c>
       <c r="F160" t="s">
         <v>189</v>
@@ -3838,10 +3838,10 @@
         <v>184</v>
       </c>
       <c r="D161" t="n">
-        <v>10.384297226497997</v>
+        <v>10.366507386852527</v>
       </c>
       <c r="E161" t="n">
-        <v>2.6604960852060886</v>
+        <v>2.629590973637306</v>
       </c>
       <c r="F161" t="s">
         <v>189</v>
@@ -3858,10 +3858,10 @@
         <v>184</v>
       </c>
       <c r="D162" t="n">
-        <v>20.811669566398642</v>
+        <v>20.655717652126683</v>
       </c>
       <c r="E162" t="n">
-        <v>5.275961000931548</v>
+        <v>5.223478042920827</v>
       </c>
       <c r="F162" t="s">
         <v>189</v>
@@ -3878,10 +3878,10 @@
         <v>182</v>
       </c>
       <c r="D163" t="n">
-        <v>47.543773753519396</v>
+        <v>47.60869137138192</v>
       </c>
       <c r="E163" t="n">
-        <v>8.167341650996331</v>
+        <v>8.115193365790436</v>
       </c>
       <c r="F163" t="s">
         <v>189</v>
@@ -3898,10 +3898,10 @@
         <v>182</v>
       </c>
       <c r="D164" t="n">
-        <v>47.66140829954973</v>
+        <v>47.523067685278015</v>
       </c>
       <c r="E164" t="n">
-        <v>8.083794177201124</v>
+        <v>8.175917728784677</v>
       </c>
       <c r="F164" t="s">
         <v>189</v>
@@ -3918,10 +3918,10 @@
         <v>182</v>
       </c>
       <c r="D165" t="n">
-        <v>47.53723936864734</v>
+        <v>47.50733987919468</v>
       </c>
       <c r="E165" t="n">
-        <v>8.130489913577064</v>
+        <v>8.170770691341833</v>
       </c>
       <c r="F165" t="s">
         <v>189</v>
@@ -3938,10 +3938,10 @@
         <v>182</v>
       </c>
       <c r="D166" t="n">
-        <v>46.71207672154662</v>
+        <v>46.61326555503776</v>
       </c>
       <c r="E166" t="n">
-        <v>8.061272354661774</v>
+        <v>8.092752534665651</v>
       </c>
       <c r="F166" t="s">
         <v>189</v>
@@ -3958,10 +3958,10 @@
         <v>182</v>
       </c>
       <c r="D167" t="n">
-        <v>54.35122926773359</v>
+        <v>54.192988525148905</v>
       </c>
       <c r="E167" t="n">
-        <v>9.163670277940906</v>
+        <v>9.195634184505353</v>
       </c>
       <c r="F167" t="s">
         <v>189</v>
@@ -3978,10 +3978,10 @@
         <v>182</v>
       </c>
       <c r="D168" t="n">
-        <v>55.35049969019408</v>
+        <v>55.392074158396795</v>
       </c>
       <c r="E168" t="n">
-        <v>9.430466396574834</v>
+        <v>9.52930720689489</v>
       </c>
       <c r="F168" t="s">
         <v>189</v>
@@ -3998,10 +3998,10 @@
         <v>182</v>
       </c>
       <c r="D169" t="n">
-        <v>54.227466180958565</v>
+        <v>54.074168901722395</v>
       </c>
       <c r="E169" t="n">
-        <v>9.150968657558515</v>
+        <v>9.215590881086085</v>
       </c>
       <c r="F169" t="s">
         <v>189</v>

</xml_diff>